<commit_message>
working on 2026 analyses
</commit_message>
<xml_diff>
--- a/data/mesquite_proximity_fall2026.xlsx
+++ b/data/mesquite_proximity_fall2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernbromley/Desktop/AVCA_BANWR/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EDC4CC-61AD-E44B-9918-39290EDDBA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB154ABF-110A-C345-A904-BC76CC853E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" xr2:uid="{B862D82C-49C1-F543-9C47-75B7F00BA096}"/>
   </bookViews>
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFF12CE4-99FC-884B-8386-7E80CE8B8E93}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -708,6 +708,270 @@
         <v>97</v>
       </c>
     </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>10</v>
+      </c>
+      <c r="B27">
+        <v>5</v>
+      </c>
+      <c r="C27">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>79</v>
+      </c>
+      <c r="B28">
+        <v>3.3</v>
+      </c>
+      <c r="C28">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <v>1.8</v>
+      </c>
+      <c r="C29">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>16</v>
+      </c>
+      <c r="B30">
+        <v>4.8</v>
+      </c>
+      <c r="C30">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>23</v>
+      </c>
+      <c r="B31">
+        <v>2.4</v>
+      </c>
+      <c r="C31">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>12</v>
+      </c>
+      <c r="B32">
+        <v>5.6</v>
+      </c>
+      <c r="C32">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>52</v>
+      </c>
+      <c r="B33">
+        <v>4.2</v>
+      </c>
+      <c r="C33">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>54</v>
+      </c>
+      <c r="B34">
+        <v>4.7</v>
+      </c>
+      <c r="C34">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>62</v>
+      </c>
+      <c r="B35">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C35">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>98</v>
+      </c>
+      <c r="B36">
+        <v>3.1</v>
+      </c>
+      <c r="C36">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>70</v>
+      </c>
+      <c r="B37">
+        <v>1.4</v>
+      </c>
+      <c r="C37">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>86</v>
+      </c>
+      <c r="B38">
+        <v>7.5</v>
+      </c>
+      <c r="C38">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>7.6</v>
+      </c>
+      <c r="C39">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>5</v>
+      </c>
+      <c r="B40">
+        <v>7.1</v>
+      </c>
+      <c r="C40">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>81</v>
+      </c>
+      <c r="B41">
+        <v>3.9</v>
+      </c>
+      <c r="C41">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>28</v>
+      </c>
+      <c r="B42">
+        <v>3.4</v>
+      </c>
+      <c r="C42">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>36</v>
+      </c>
+      <c r="B43">
+        <v>2.75</v>
+      </c>
+      <c r="C43">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>58</v>
+      </c>
+      <c r="B44">
+        <v>3.25</v>
+      </c>
+      <c r="C44">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>73</v>
+      </c>
+      <c r="B45">
+        <v>1.6</v>
+      </c>
+      <c r="C45">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>75</v>
+      </c>
+      <c r="B46">
+        <v>1.5</v>
+      </c>
+      <c r="C46">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>42</v>
+      </c>
+      <c r="B47">
+        <v>1.7</v>
+      </c>
+      <c r="C47">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>6</v>
+      </c>
+      <c r="B48">
+        <v>1.7</v>
+      </c>
+      <c r="C48">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>1</v>
+      </c>
+      <c r="B49">
+        <v>2.5</v>
+      </c>
+      <c r="C49">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>100</v>
+      </c>
+      <c r="B50">
+        <v>1.7</v>
+      </c>
+      <c r="C50">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>